<commit_message>
moved connectors further over the board outline to fit them better into the housing of the pcb. regenerated outputjob files, added housing CAD data
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
+++ b/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_torque_box\Project Outputs for uz_per_torque_box\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D38B664C-F9E3-4646-A790-07507AE4F77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF367EA0-3033-4CAA-9D98-7F4371DAE42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" xr2:uid="{D254624D-B5F4-452F-BAD6-1683F1703D90}"/>
+    <workbookView xWindow="67290" yWindow="-2325" windowWidth="19125" windowHeight="10035" xr2:uid="{77662519-F4E0-4121-B91C-C730E606813D}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_torque_box(Defau" sheetId="1" r:id="rId1"/>
@@ -752,7 +752,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD086BD-609A-4EE1-B125-230C06DAAB6D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A9911E-DC52-47EF-8BD5-32E76A68ED7D}">
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
updated pcb project with new 3d body for dsub15. recreated step file and updated cad project. updated outputjobfiles
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
+++ b/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_torque_box\Project Outputs for uz_per_torque_box\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF367EA0-3033-4CAA-9D98-7F4371DAE42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EA4D605-756F-44E4-956D-CE4B37B4A598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67290" yWindow="-2325" windowWidth="19125" windowHeight="10035" xr2:uid="{77662519-F4E0-4121-B91C-C730E606813D}"/>
+    <workbookView xWindow="38925" yWindow="135" windowWidth="19125" windowHeight="10035" xr2:uid="{1F1528EC-AD57-4C16-800D-EA0F84B51F4F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_torque_box(Defau" sheetId="1" r:id="rId1"/>
@@ -752,7 +752,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A9911E-DC52-47EF-8BD5-32E76A68ED7D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799A3F23-F085-4203-8F2D-AEEAA90A1453}">
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
moved Samtec IPL 1mm inwards, for hopefully better mountability in the housing. exported step, regenerated outputjob
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
+++ b/Project Outputs for uz_per_torque_box/Rev01/BOM/BOM_JLC-uz_per_torque_box(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_torque_box\Project Outputs for uz_per_torque_box\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EA4D605-756F-44E4-956D-CE4B37B4A598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7E23810-ED06-45D0-9E05-865D043BFB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38925" yWindow="135" windowWidth="19125" windowHeight="10035" xr2:uid="{1F1528EC-AD57-4C16-800D-EA0F84B51F4F}"/>
+    <workbookView xWindow="38925" yWindow="135" windowWidth="19125" windowHeight="10035" xr2:uid="{FC3DBFCE-7EE3-42A4-A146-41CE7DA3C43B}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_torque_box(Defau" sheetId="1" r:id="rId1"/>
@@ -752,7 +752,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799A3F23-F085-4203-8F2D-AEEAA90A1453}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F6B8435-3D0D-449F-AEE6-4A5FF8FCFF14}">
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>